<commit_message>
docs: update DEVLOG and README with Phase 16-20 (order history, void, stock UI, is_sellable migration)
</commit_message>
<xml_diff>
--- a/data/master_menu.xlsx
+++ b/data/master_menu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Download\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS\pos-cak-kino\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A79638-24A0-4213-85CE-CA86F5AB6D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D97696-E093-45F0-A348-917AB26B8AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,15 @@
     <sheet name="OpeningStock" sheetId="6" r:id="rId6"/>
     <sheet name="PaketComponents" sheetId="7" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Menus!$A$1:$E$39</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="161">
   <si>
     <t>Master Menu — Penyetan Sedap Malam Cak Kino</t>
   </si>
@@ -503,6 +506,12 @@
   </si>
   <si>
     <t>qty_per_paket</t>
+  </si>
+  <si>
+    <t>is_sellable</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
 </sst>
 </file>
@@ -1230,7 +1239,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1240,7 +1249,7 @@
     <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>61</v>
       </c>
@@ -1256,8 +1265,11 @@
       <c r="E1" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>65</v>
       </c>
@@ -1274,7 +1286,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>69</v>
       </c>
@@ -1291,7 +1303,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>71</v>
       </c>
@@ -1308,7 +1320,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>73</v>
       </c>
@@ -1325,7 +1337,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>75</v>
       </c>
@@ -1342,7 +1354,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>77</v>
       </c>
@@ -1359,7 +1371,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>79</v>
       </c>
@@ -1376,7 +1388,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>81</v>
       </c>
@@ -1393,7 +1405,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>82</v>
       </c>
@@ -1410,7 +1422,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>83</v>
       </c>
@@ -1427,7 +1439,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>84</v>
       </c>
@@ -1443,8 +1455,11 @@
       <c r="E12" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>85</v>
       </c>
@@ -1460,8 +1475,11 @@
       <c r="E13" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>87</v>
       </c>
@@ -1477,8 +1495,11 @@
       <c r="E14" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>89</v>
       </c>
@@ -1494,8 +1515,11 @@
       <c r="E15" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F15" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>91</v>
       </c>
@@ -1511,8 +1535,11 @@
       <c r="E16" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>93</v>
       </c>
@@ -1528,8 +1555,11 @@
       <c r="E17" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F17" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>95</v>
       </c>
@@ -1545,8 +1575,11 @@
       <c r="E18" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>97</v>
       </c>
@@ -1562,8 +1595,11 @@
       <c r="E19" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>99</v>
       </c>
@@ -1579,8 +1615,11 @@
       <c r="E20" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>101</v>
       </c>
@@ -1596,8 +1635,11 @@
       <c r="E21" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>103</v>
       </c>
@@ -1613,8 +1655,11 @@
       <c r="E22" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>105</v>
       </c>
@@ -1630,8 +1675,11 @@
       <c r="E23" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>107</v>
       </c>
@@ -1647,8 +1695,11 @@
       <c r="E24" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>109</v>
       </c>
@@ -1664,8 +1715,11 @@
       <c r="E25" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F25" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>111</v>
       </c>
@@ -1681,8 +1735,11 @@
       <c r="E26" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F26" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>113</v>
       </c>
@@ -1698,8 +1755,11 @@
       <c r="E27" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>115</v>
       </c>
@@ -1715,8 +1775,11 @@
       <c r="E28" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
         <v>117</v>
       </c>
@@ -1732,8 +1795,11 @@
       <c r="E29" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F29" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>119</v>
       </c>
@@ -1749,8 +1815,11 @@
       <c r="E30" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F30" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>121</v>
       </c>
@@ -1766,8 +1835,11 @@
       <c r="E31" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F31" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>123</v>
       </c>
@@ -1783,8 +1855,11 @@
       <c r="E32" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F32" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>125</v>
       </c>
@@ -1800,8 +1875,11 @@
       <c r="E33" s="8" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F33" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>127</v>
       </c>
@@ -1817,8 +1895,11 @@
       <c r="E34" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F34" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
         <v>130</v>
       </c>
@@ -1834,8 +1915,11 @@
       <c r="E35" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F35" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>132</v>
       </c>
@@ -1851,8 +1935,11 @@
       <c r="E36" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F36" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
         <v>134</v>
       </c>
@@ -1868,8 +1955,11 @@
       <c r="E37" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F37" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
         <v>136</v>
       </c>
@@ -1885,8 +1975,11 @@
       <c r="E38" s="7" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F38" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>138</v>
       </c>
@@ -1900,6 +1993,9 @@
         <v>129</v>
       </c>
       <c r="E39" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>68</v>
       </c>
     </row>
@@ -2551,7 +2647,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2571,39 +2667,255 @@
         <v>65</v>
       </c>
       <c r="B2" s="7">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B3" s="7">
-        <v>20</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B4" s="7">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="8">
-        <v>30</v>
+      <c r="A5" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="7">
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B11" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" s="7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B23" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B24" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="7">
-        <v>40</v>
+      <c r="B28" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B29" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B31" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B32" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B33" s="7">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(menu): add is_sellable flag for base-unit items
</commit_message>
<xml_diff>
--- a/data/master_menu.xlsx
+++ b/data/master_menu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS\pos-cak-kino\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D97696-E093-45F0-A348-917AB26B8AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874C56B5-D9F0-4A72-9C70-A01B2B0971A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="161">
   <si>
     <t>Master Menu — Penyetan Sedap Malam Cak Kino</t>
   </si>
@@ -1247,6 +1247,7 @@
     <col min="3" max="3" width="40" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -1285,6 +1286,9 @@
       <c r="E2" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F2" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
@@ -1302,6 +1306,9 @@
       <c r="E3" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F3" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
@@ -1319,6 +1326,9 @@
       <c r="E4" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F4" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -1336,6 +1346,9 @@
       <c r="E5" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F5" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
@@ -1353,6 +1366,9 @@
       <c r="E6" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F6" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
@@ -1370,6 +1386,9 @@
       <c r="E7" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F7" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -1387,6 +1406,9 @@
       <c r="E8" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F8" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
@@ -1404,6 +1426,9 @@
       <c r="E9" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F9" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
@@ -1421,6 +1446,9 @@
       <c r="E10" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="F10" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
@@ -1436,6 +1464,9 @@
         <v>67</v>
       </c>
       <c r="E11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>68</v>
       </c>
     </row>

</xml_diff>